<commit_message>
Pushing Evo stuff. I really should make separate branches...
</commit_message>
<xml_diff>
--- a/EvolutionPOC/LangMod/EN/SourceSheet.xlsx
+++ b/EvolutionPOC/LangMod/EN/SourceSheet.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="143">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -340,6 +340,9 @@
     <t xml:space="preserve">testchara_evo_stage1</t>
   </si>
   <si>
+    <t xml:space="preserve">*r</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dragon Miko</t>
   </si>
   <si>
@@ -376,7 +379,7 @@
     <t xml:space="preserve">Awakened Dragon Miko</t>
   </si>
   <si>
-    <t xml:space="preserve">evolve#testchara_evo_stage3#evolution_heart_b</t>
+    <t xml:space="preserve">evolve#testchara_evo_stage3#evolution_heart_b,noEgg</t>
   </si>
   <si>
     <t xml:space="preserve">testchara_evo_stage3</t>
@@ -385,6 +388,9 @@
     <t xml:space="preserve">Water Goddess</t>
   </si>
   <si>
+    <t xml:space="preserve">noEgg</t>
+  </si>
+  <si>
     <t xml:space="preserve">group</t>
   </si>
   <si>
@@ -415,7 +421,16 @@
     <t xml:space="preserve">Good</t>
   </si>
   <si>
-    <t xml:space="preserve">#1 has evolved into #2!</t>
+    <t xml:space="preserve">#1 the #2 has evolved into #3!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">noEgg_Tag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">negative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This character cannot produce eggs.</t>
   </si>
   <si>
     <t xml:space="preserve">evolutionConfirmation</t>
@@ -430,7 +445,7 @@
     <t xml:space="preserve">evolveChara</t>
   </si>
   <si>
-    <t xml:space="preserve">Evolve into #1</t>
+    <t xml:space="preserve">Evolve into #1.</t>
   </si>
   <si>
     <t xml:space="preserve">evolutionAffinityRequirementNotMet</t>
@@ -448,7 +463,7 @@
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="@"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -527,6 +542,11 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FFD0D0D0"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
@@ -572,6 +592,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFC9A26D"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
     <font>
       <sz val="10"/>
@@ -647,7 +673,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -736,31 +762,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -768,11 +802,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -788,7 +822,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3144,16 +3178,18 @@
         <v>7869001</v>
       </c>
       <c r="C4" s="14"/>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="1" t="s">
         <v>105</v>
       </c>
       <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
+      <c r="F4" s="7" t="s">
+        <v>106</v>
+      </c>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
       <c r="I4" s="7"/>
       <c r="J4" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
@@ -3162,7 +3198,7 @@
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P4" s="7" t="n">
         <v>10</v>
@@ -3174,29 +3210,29 @@
         <v>4</v>
       </c>
       <c r="S4" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="T4" s="7"/>
       <c r="U4" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="V4" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="W4" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="X4" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Y4" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Z4" s="7"/>
       <c r="AA4" s="7"/>
       <c r="AB4" s="7"/>
       <c r="AC4" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AD4" s="7"/>
       <c r="AE4" s="7" t="s">
@@ -3225,22 +3261,24 @@
     </row>
     <row r="5" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B5" s="15" t="n">
         <v>7869002</v>
       </c>
       <c r="C5" s="7"/>
-      <c r="D5" s="7" t="s">
-        <v>116</v>
+      <c r="D5" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="E5" s="14"/>
-      <c r="F5" s="7"/>
+      <c r="F5" s="7" t="s">
+        <v>117</v>
+      </c>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
       <c r="I5" s="7"/>
       <c r="J5" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
@@ -3249,7 +3287,7 @@
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P5" s="7" t="n">
         <v>20</v>
@@ -3261,29 +3299,29 @@
         <v>4</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="T5" s="7"/>
       <c r="U5" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="V5" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="W5" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="X5" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Y5" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Z5" s="7"/>
       <c r="AA5" s="7"/>
       <c r="AB5" s="7"/>
       <c r="AC5" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AD5" s="7"/>
       <c r="AE5" s="7" t="s">
@@ -3312,22 +3350,24 @@
     </row>
     <row r="6" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B6" s="15" t="n">
         <v>7869003</v>
       </c>
       <c r="C6" s="14"/>
-      <c r="D6" s="7" t="s">
-        <v>119</v>
+      <c r="D6" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
+      <c r="F6" s="7" t="s">
+        <v>120</v>
+      </c>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
       <c r="J6" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K6" s="7"/>
       <c r="L6" s="7"/>
@@ -3336,7 +3376,7 @@
       </c>
       <c r="N6" s="7"/>
       <c r="O6" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P6" s="7" t="n">
         <v>30</v>
@@ -3348,27 +3388,29 @@
         <v>4</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="T6" s="7"/>
-      <c r="U6" s="7"/>
+      <c r="U6" s="18" t="s">
+        <v>121</v>
+      </c>
       <c r="V6" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="W6" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="X6" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
       <c r="AB6" s="7"/>
       <c r="AC6" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AD6" s="7"/>
       <c r="AE6" s="7" t="s">
@@ -3406,7 +3448,7 @@
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
       <c r="S7" s="7"/>
-      <c r="V7" s="18"/>
+      <c r="V7" s="19"/>
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="7"/>
@@ -3420,9 +3462,9 @@
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7"/>
       <c r="B8" s="15"/>
-      <c r="C8" s="19"/>
+      <c r="C8" s="20"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="20"/>
+      <c r="E8" s="21"/>
       <c r="F8" s="7"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
@@ -3438,7 +3480,7 @@
       <c r="R8" s="7"/>
       <c r="S8" s="7"/>
       <c r="T8" s="1"/>
-      <c r="V8" s="18"/>
+      <c r="V8" s="19"/>
       <c r="W8" s="1"/>
       <c r="X8" s="13"/>
       <c r="Y8" s="7"/>
@@ -3476,7 +3518,7 @@
       <c r="Q9" s="7"/>
       <c r="R9" s="7"/>
       <c r="S9" s="7"/>
-      <c r="V9" s="18"/>
+      <c r="V9" s="19"/>
       <c r="W9" s="1"/>
       <c r="X9" s="1"/>
       <c r="Y9" s="1"/>
@@ -3496,7 +3538,7 @@
       <c r="Q10" s="7"/>
       <c r="R10" s="7"/>
       <c r="S10" s="7"/>
-      <c r="V10" s="18"/>
+      <c r="V10" s="19"/>
       <c r="W10" s="1"/>
       <c r="X10" s="1"/>
       <c r="Y10" s="1"/>
@@ -3516,7 +3558,7 @@
       <c r="Q11" s="7"/>
       <c r="R11" s="7"/>
       <c r="S11" s="7"/>
-      <c r="V11" s="18"/>
+      <c r="V11" s="19"/>
       <c r="W11" s="1"/>
       <c r="X11" s="1"/>
       <c r="Y11" s="1"/>
@@ -3536,7 +3578,7 @@
       <c r="Q12" s="7"/>
       <c r="R12" s="7"/>
       <c r="S12" s="7"/>
-      <c r="V12" s="18"/>
+      <c r="V12" s="19"/>
       <c r="W12" s="1"/>
       <c r="X12" s="1"/>
       <c r="Y12" s="1"/>
@@ -3580,7 +3622,7 @@
       <c r="R14" s="1"/>
       <c r="S14" s="7"/>
       <c r="W14" s="1"/>
-      <c r="X14" s="21"/>
+      <c r="X14" s="22"/>
       <c r="Y14" s="7"/>
       <c r="Z14" s="1"/>
       <c r="AB14" s="7"/>
@@ -3702,7 +3744,7 @@
     </row>
     <row r="20" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="15"/>
-      <c r="C20" s="22"/>
+      <c r="C20" s="23"/>
       <c r="D20" s="7"/>
       <c r="J20" s="7"/>
       <c r="M20" s="1"/>
@@ -3723,7 +3765,7 @@
     </row>
     <row r="21" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="15"/>
-      <c r="C21" s="22"/>
+      <c r="C21" s="23"/>
       <c r="J21" s="7"/>
       <c r="M21" s="1"/>
       <c r="P21" s="1"/>
@@ -3741,7 +3783,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="15"/>
-      <c r="C22" s="22"/>
+      <c r="C22" s="23"/>
       <c r="J22" s="7"/>
       <c r="M22" s="1"/>
       <c r="P22" s="1"/>
@@ -3760,7 +3802,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="15"/>
-      <c r="C23" s="22"/>
+      <c r="C23" s="23"/>
       <c r="J23" s="7"/>
       <c r="M23" s="1"/>
       <c r="P23" s="1"/>
@@ -3779,7 +3821,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="15"/>
-      <c r="C24" s="22"/>
+      <c r="C24" s="23"/>
       <c r="J24" s="7"/>
       <c r="M24" s="1"/>
       <c r="P24" s="1"/>
@@ -3798,7 +3840,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="15"/>
-      <c r="C25" s="22"/>
+      <c r="C25" s="23"/>
       <c r="J25" s="7"/>
       <c r="M25" s="1"/>
       <c r="P25" s="1"/>
@@ -3817,7 +3859,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="15"/>
-      <c r="C26" s="22"/>
+      <c r="C26" s="23"/>
       <c r="J26" s="7"/>
       <c r="M26" s="1"/>
       <c r="P26" s="1"/>
@@ -3836,7 +3878,7 @@
     </row>
     <row r="27" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="15"/>
-      <c r="C27" s="22"/>
+      <c r="C27" s="23"/>
       <c r="J27" s="7"/>
       <c r="M27" s="1"/>
       <c r="P27" s="1"/>
@@ -3855,7 +3897,7 @@
     </row>
     <row r="28" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="15"/>
-      <c r="C28" s="22"/>
+      <c r="C28" s="23"/>
       <c r="J28" s="7"/>
       <c r="M28" s="1"/>
       <c r="P28" s="1"/>
@@ -3873,7 +3915,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="15"/>
-      <c r="C29" s="22"/>
+      <c r="C29" s="23"/>
       <c r="J29" s="7"/>
       <c r="M29" s="1"/>
       <c r="P29" s="1"/>
@@ -3927,7 +3969,7 @@
       <c r="AL31" s="1"/>
     </row>
     <row r="32" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="23"/>
+      <c r="A32" s="24"/>
       <c r="B32" s="15"/>
       <c r="C32" s="7"/>
       <c r="J32" s="7"/>
@@ -4367,96 +4409,96 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="24" t="s">
-        <v>120</v>
-      </c>
-      <c r="D1" s="24" t="s">
-        <v>121</v>
-      </c>
-      <c r="E1" s="24" t="s">
+      <c r="C1" s="25" t="s">
         <v>122</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="D1" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="E1" s="25" t="s">
         <v>124</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="F1" s="25" t="s">
         <v>125</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="G1" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="25"/>
-      <c r="R1" s="25"/>
-      <c r="S1" s="25"/>
-      <c r="T1" s="25"/>
-      <c r="U1" s="25"/>
-      <c r="V1" s="25"/>
-      <c r="W1" s="25"/>
-      <c r="X1" s="25"/>
-      <c r="Y1" s="25"/>
-      <c r="Z1" s="25"/>
+      <c r="H1" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="I1" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
+      <c r="Q1" s="26"/>
+      <c r="R1" s="26"/>
+      <c r="S1" s="26"/>
+      <c r="T1" s="26"/>
+      <c r="U1" s="26"/>
+      <c r="V1" s="26"/>
+      <c r="W1" s="26"/>
+      <c r="X1" s="26"/>
+      <c r="Y1" s="26"/>
+      <c r="Z1" s="26"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="D2" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="E2" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="G2" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="H2" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="I2" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="25"/>
-      <c r="P2" s="25"/>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
-      <c r="S2" s="25"/>
-      <c r="T2" s="25"/>
-      <c r="U2" s="25"/>
-      <c r="V2" s="25"/>
-      <c r="W2" s="25"/>
-      <c r="X2" s="25"/>
-      <c r="Y2" s="25"/>
-      <c r="Z2" s="25"/>
+      <c r="A2" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="G2" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
+      <c r="R2" s="26"/>
+      <c r="S2" s="26"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
+      <c r="V2" s="26"/>
+      <c r="W2" s="26"/>
+      <c r="X2" s="26"/>
+      <c r="Y2" s="26"/>
+      <c r="Z2" s="26"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7"/>
@@ -4468,43 +4510,51 @@
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
-      <c r="M3" s="25"/>
-      <c r="N3" s="25"/>
-      <c r="O3" s="25"/>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="25"/>
-      <c r="R3" s="25"/>
-      <c r="S3" s="25"/>
-      <c r="T3" s="25"/>
-      <c r="U3" s="25"/>
-      <c r="V3" s="25"/>
-      <c r="W3" s="25"/>
-      <c r="X3" s="25"/>
-      <c r="Y3" s="25"/>
-      <c r="Z3" s="25"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26"/>
+      <c r="T3" s="26"/>
+      <c r="U3" s="26"/>
+      <c r="V3" s="26"/>
+      <c r="W3" s="26"/>
+      <c r="X3" s="26"/>
+      <c r="Y3" s="26"/>
+      <c r="Z3" s="26"/>
     </row>
     <row r="4" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="D4" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="E4" s="24" t="s">
         <v>129</v>
       </c>
+      <c r="D4" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>131</v>
+      </c>
       <c r="I4" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26"/>
+      <c r="A5" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="26"/>
+      <c r="A6" s="28"/>
       <c r="B6" s="1"/>
       <c r="D6" s="1"/>
     </row>
@@ -4544,112 +4594,112 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="27" t="s">
-        <v>125</v>
-      </c>
-      <c r="D1" s="27" t="s">
-        <v>126</v>
-      </c>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="25"/>
-      <c r="R1" s="25"/>
-      <c r="S1" s="25"/>
-      <c r="T1" s="25"/>
-      <c r="U1" s="25"/>
-      <c r="V1" s="25"/>
-      <c r="W1" s="25"/>
-      <c r="X1" s="25"/>
-      <c r="Y1" s="25"/>
+      <c r="C1" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
+      <c r="Q1" s="26"/>
+      <c r="R1" s="26"/>
+      <c r="S1" s="26"/>
+      <c r="T1" s="26"/>
+      <c r="U1" s="26"/>
+      <c r="V1" s="26"/>
+      <c r="W1" s="26"/>
+      <c r="X1" s="26"/>
+      <c r="Y1" s="26"/>
     </row>
     <row r="2" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="25"/>
-      <c r="P2" s="25"/>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
-      <c r="S2" s="25"/>
-      <c r="T2" s="25"/>
-      <c r="U2" s="25"/>
-      <c r="V2" s="25"/>
-      <c r="W2" s="25"/>
-      <c r="X2" s="25"/>
-      <c r="Y2" s="25"/>
+      <c r="A2" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
+      <c r="R2" s="26"/>
+      <c r="S2" s="26"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
+      <c r="V2" s="26"/>
+      <c r="W2" s="26"/>
+      <c r="X2" s="26"/>
+      <c r="Y2" s="26"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="25"/>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
-      <c r="M3" s="25"/>
-      <c r="N3" s="25"/>
-      <c r="O3" s="25"/>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="25"/>
-      <c r="R3" s="25"/>
-      <c r="S3" s="25"/>
-      <c r="T3" s="25"/>
-      <c r="U3" s="25"/>
-      <c r="V3" s="25"/>
-      <c r="W3" s="25"/>
-      <c r="X3" s="25"/>
-      <c r="Y3" s="25"/>
+      <c r="A3" s="26"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26"/>
+      <c r="T3" s="26"/>
+      <c r="U3" s="26"/>
+      <c r="V3" s="26"/>
+      <c r="W3" s="26"/>
+      <c r="X3" s="26"/>
+      <c r="Y3" s="26"/>
     </row>
     <row r="4" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
-        <v>131</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>132</v>
-      </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29" t="s">
-        <v>133</v>
+      <c r="A4" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31" t="s">
+        <v>138</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
@@ -4674,15 +4724,15 @@
       <c r="Y4" s="7"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="30" t="s">
-        <v>134</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>132</v>
-      </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31" t="s">
-        <v>135</v>
+      <c r="A5" s="32" t="s">
+        <v>139</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>137</v>
+      </c>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33" t="s">
+        <v>140</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
@@ -4707,15 +4757,15 @@
       <c r="Y5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="30" t="s">
-        <v>136</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>132</v>
-      </c>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31" t="s">
+      <c r="A6" s="32" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6" s="33" t="s">
         <v>137</v>
+      </c>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33" t="s">
+        <v>142</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
@@ -4740,10 +4790,10 @@
       <c r="Y6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="32"/>
-      <c r="B7" s="31"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
+      <c r="A7" s="34"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -4767,10 +4817,10 @@
       <c r="Y7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29"/>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
+      <c r="A8" s="31"/>
+      <c r="B8" s="31"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
@@ -4794,10 +4844,10 @@
       <c r="Y8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29"/>
-      <c r="B9" s="29"/>
-      <c r="C9" s="29"/>
-      <c r="D9" s="29"/>
+      <c r="A9" s="31"/>
+      <c r="B9" s="31"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
@@ -4821,10 +4871,10 @@
       <c r="Y9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
+      <c r="A10" s="31"/>
+      <c r="B10" s="31"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
@@ -4848,10 +4898,10 @@
       <c r="Y10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29"/>
-      <c r="B11" s="29"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29"/>
+      <c r="A11" s="31"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
@@ -4875,10 +4925,10 @@
       <c r="Y11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="29"/>
-      <c r="D12" s="29"/>
+      <c r="A12" s="31"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
@@ -4902,10 +4952,10 @@
       <c r="Y12" s="7"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29"/>
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
+      <c r="A13" s="31"/>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
@@ -4929,10 +4979,10 @@
       <c r="Y13" s="7"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29"/>
-      <c r="B14" s="29"/>
-      <c r="C14" s="29"/>
-      <c r="D14" s="29"/>
+      <c r="A14" s="31"/>
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
@@ -4956,10 +5006,10 @@
       <c r="Y14" s="7"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="29"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
+      <c r="A15" s="31"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
@@ -4983,10 +5033,10 @@
       <c r="Y15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
+      <c r="A16" s="31"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
@@ -5010,10 +5060,10 @@
       <c r="Y16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
+      <c r="A17" s="31"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
@@ -5037,10 +5087,10 @@
       <c r="Y17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
+      <c r="A18" s="31"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
@@ -5064,10 +5114,10 @@
       <c r="Y18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
+      <c r="A19" s="31"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
@@ -5091,10 +5141,10 @@
       <c r="Y19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29"/>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
+      <c r="A20" s="31"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
@@ -5118,16 +5168,16 @@
       <c r="Y20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="29"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
+      <c r="A21" s="31"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
+      <c r="A22" s="31"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
@@ -5151,10 +5201,10 @@
       <c r="Y22" s="7"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="29"/>
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
+      <c r="A23" s="31"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
@@ -5178,10 +5228,10 @@
       <c r="Y23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="29"/>
-      <c r="B24" s="29"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
+      <c r="A24" s="31"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
       <c r="G24" s="7"/>
@@ -5205,10 +5255,10 @@
       <c r="Y24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29"/>
-      <c r="B25" s="29"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
+      <c r="A25" s="31"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
@@ -5232,10 +5282,10 @@
       <c r="Y25" s="1"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
+      <c r="A26" s="31"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
@@ -5259,10 +5309,10 @@
       <c r="Y26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="29"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
+      <c r="A27" s="31"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
@@ -5286,10 +5336,10 @@
       <c r="Y27" s="7"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
+      <c r="A28" s="31"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
       <c r="E28" s="7"/>
       <c r="F28" s="7"/>
       <c r="G28" s="7"/>
@@ -5313,10 +5363,10 @@
       <c r="Y28" s="7"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29"/>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
+      <c r="A29" s="31"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
@@ -5340,10 +5390,10 @@
       <c r="Y29" s="7"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="29"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
+      <c r="A30" s="31"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
       <c r="E30" s="7"/>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
@@ -5367,10 +5417,10 @@
       <c r="Y30" s="7"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="29"/>
-      <c r="B31" s="29"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
+      <c r="A31" s="31"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
@@ -5394,37 +5444,37 @@
       <c r="Y31" s="7"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="29"/>
-      <c r="B32" s="29"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="33"/>
-      <c r="G32" s="33"/>
-      <c r="H32" s="33"/>
-      <c r="I32" s="33"/>
-      <c r="J32" s="33"/>
-      <c r="K32" s="33"/>
-      <c r="L32" s="33"/>
-      <c r="M32" s="33"/>
-      <c r="N32" s="33"/>
-      <c r="O32" s="33"/>
-      <c r="P32" s="33"/>
-      <c r="Q32" s="33"/>
-      <c r="R32" s="33"/>
-      <c r="S32" s="33"/>
-      <c r="T32" s="33"/>
-      <c r="U32" s="33"/>
-      <c r="V32" s="33"/>
-      <c r="W32" s="33"/>
-      <c r="X32" s="33"/>
-      <c r="Y32" s="33"/>
+      <c r="A32" s="31"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="35"/>
+      <c r="F32" s="35"/>
+      <c r="G32" s="35"/>
+      <c r="H32" s="35"/>
+      <c r="I32" s="35"/>
+      <c r="J32" s="35"/>
+      <c r="K32" s="35"/>
+      <c r="L32" s="35"/>
+      <c r="M32" s="35"/>
+      <c r="N32" s="35"/>
+      <c r="O32" s="35"/>
+      <c r="P32" s="35"/>
+      <c r="Q32" s="35"/>
+      <c r="R32" s="35"/>
+      <c r="S32" s="35"/>
+      <c r="T32" s="35"/>
+      <c r="U32" s="35"/>
+      <c r="V32" s="35"/>
+      <c r="W32" s="35"/>
+      <c r="X32" s="35"/>
+      <c r="Y32" s="35"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="29"/>
-      <c r="B33" s="29"/>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29"/>
+      <c r="A33" s="31"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
@@ -5448,10 +5498,10 @@
       <c r="Y33" s="1"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="29"/>
-      <c r="B34" s="29"/>
-      <c r="C34" s="29"/>
-      <c r="D34" s="29"/>
+      <c r="A34" s="31"/>
+      <c r="B34" s="31"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
@@ -5475,10 +5525,10 @@
       <c r="Y34" s="1"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="29"/>
-      <c r="B35" s="29"/>
-      <c r="C35" s="29"/>
-      <c r="D35" s="29"/>
+      <c r="A35" s="31"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="31"/>
+      <c r="D35" s="31"/>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
@@ -5502,10 +5552,10 @@
       <c r="Y35" s="1"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="29"/>
-      <c r="B36" s="29"/>
-      <c r="C36" s="29"/>
-      <c r="D36" s="29"/>
+      <c r="A36" s="31"/>
+      <c r="B36" s="31"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
@@ -5529,10 +5579,10 @@
       <c r="Y36" s="1"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="29"/>
-      <c r="B37" s="29"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="34"/>
+      <c r="A37" s="31"/>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="36"/>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
@@ -5556,178 +5606,178 @@
       <c r="Y37" s="1"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="29"/>
-      <c r="B38" s="29"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="34"/>
+      <c r="A38" s="31"/>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="36"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="29"/>
-      <c r="B39" s="29"/>
-      <c r="C39" s="29"/>
-      <c r="D39" s="34"/>
+      <c r="A39" s="31"/>
+      <c r="B39" s="31"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="36"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="29"/>
-      <c r="B40" s="29"/>
-      <c r="C40" s="29"/>
-      <c r="D40" s="34"/>
+      <c r="A40" s="31"/>
+      <c r="B40" s="31"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="36"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="29"/>
-      <c r="B41" s="29"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="34"/>
+      <c r="A41" s="31"/>
+      <c r="B41" s="31"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="36"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="29"/>
-      <c r="B42" s="29"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="34"/>
+      <c r="A42" s="31"/>
+      <c r="B42" s="31"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="36"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="29"/>
-      <c r="B43" s="29"/>
-      <c r="C43" s="29"/>
-      <c r="D43" s="34"/>
+      <c r="A43" s="31"/>
+      <c r="B43" s="31"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="36"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="29"/>
-      <c r="B44" s="29"/>
-      <c r="C44" s="29"/>
-      <c r="D44" s="34"/>
+      <c r="A44" s="31"/>
+      <c r="B44" s="31"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="36"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="29"/>
-      <c r="B45" s="29"/>
-      <c r="C45" s="29"/>
-      <c r="D45" s="34"/>
+      <c r="A45" s="31"/>
+      <c r="B45" s="31"/>
+      <c r="C45" s="31"/>
+      <c r="D45" s="36"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="29"/>
-      <c r="B46" s="29"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="34"/>
+      <c r="A46" s="31"/>
+      <c r="B46" s="31"/>
+      <c r="C46" s="31"/>
+      <c r="D46" s="36"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="29"/>
-      <c r="B47" s="29"/>
-      <c r="C47" s="29"/>
-      <c r="D47" s="34"/>
+      <c r="A47" s="31"/>
+      <c r="B47" s="31"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="36"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="29"/>
-      <c r="B48" s="29"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="34"/>
+      <c r="A48" s="31"/>
+      <c r="B48" s="31"/>
+      <c r="C48" s="31"/>
+      <c r="D48" s="36"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="29"/>
-      <c r="B49" s="29"/>
-      <c r="C49" s="29"/>
-      <c r="D49" s="34"/>
+      <c r="A49" s="31"/>
+      <c r="B49" s="31"/>
+      <c r="C49" s="31"/>
+      <c r="D49" s="36"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="29"/>
-      <c r="B50" s="29"/>
-      <c r="C50" s="29"/>
-      <c r="D50" s="34"/>
+      <c r="A50" s="31"/>
+      <c r="B50" s="31"/>
+      <c r="C50" s="31"/>
+      <c r="D50" s="36"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="29"/>
-      <c r="B51" s="29"/>
-      <c r="C51" s="29"/>
-      <c r="D51" s="34"/>
+      <c r="A51" s="31"/>
+      <c r="B51" s="31"/>
+      <c r="C51" s="31"/>
+      <c r="D51" s="36"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="29"/>
-      <c r="B52" s="29"/>
-      <c r="C52" s="29"/>
-      <c r="D52" s="34"/>
+      <c r="A52" s="31"/>
+      <c r="B52" s="31"/>
+      <c r="C52" s="31"/>
+      <c r="D52" s="36"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="29"/>
-      <c r="B53" s="29"/>
-      <c r="C53" s="29"/>
-      <c r="D53" s="34"/>
+      <c r="A53" s="31"/>
+      <c r="B53" s="31"/>
+      <c r="C53" s="31"/>
+      <c r="D53" s="36"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="29"/>
-      <c r="B54" s="29"/>
-      <c r="C54" s="29"/>
-      <c r="D54" s="34"/>
+      <c r="A54" s="31"/>
+      <c r="B54" s="31"/>
+      <c r="C54" s="31"/>
+      <c r="D54" s="36"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="29"/>
-      <c r="B55" s="29"/>
-      <c r="C55" s="29"/>
-      <c r="D55" s="34"/>
+      <c r="A55" s="31"/>
+      <c r="B55" s="31"/>
+      <c r="C55" s="31"/>
+      <c r="D55" s="36"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="29"/>
-      <c r="B56" s="29"/>
-      <c r="C56" s="29"/>
-      <c r="D56" s="34"/>
+      <c r="A56" s="31"/>
+      <c r="B56" s="31"/>
+      <c r="C56" s="31"/>
+      <c r="D56" s="36"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="29"/>
-      <c r="B57" s="29"/>
-      <c r="C57" s="29"/>
-      <c r="D57" s="34"/>
+      <c r="A57" s="31"/>
+      <c r="B57" s="31"/>
+      <c r="C57" s="31"/>
+      <c r="D57" s="36"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="29"/>
-      <c r="B58" s="29"/>
-      <c r="C58" s="29"/>
-      <c r="D58" s="34"/>
+      <c r="A58" s="31"/>
+      <c r="B58" s="31"/>
+      <c r="C58" s="31"/>
+      <c r="D58" s="36"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="29"/>
-      <c r="B59" s="29"/>
-      <c r="C59" s="29"/>
-      <c r="D59" s="34"/>
+      <c r="A59" s="31"/>
+      <c r="B59" s="31"/>
+      <c r="C59" s="31"/>
+      <c r="D59" s="36"/>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="29"/>
-      <c r="B60" s="29"/>
-      <c r="C60" s="29"/>
-      <c r="D60" s="34"/>
+      <c r="A60" s="31"/>
+      <c r="B60" s="31"/>
+      <c r="C60" s="31"/>
+      <c r="D60" s="36"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="29"/>
-      <c r="B61" s="29"/>
-      <c r="C61" s="29"/>
-      <c r="D61" s="34"/>
+      <c r="A61" s="31"/>
+      <c r="B61" s="31"/>
+      <c r="C61" s="31"/>
+      <c r="D61" s="36"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="29"/>
-      <c r="B62" s="29"/>
-      <c r="C62" s="29"/>
-      <c r="D62" s="34"/>
+      <c r="A62" s="31"/>
+      <c r="B62" s="31"/>
+      <c r="C62" s="31"/>
+      <c r="D62" s="36"/>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="29"/>
-      <c r="B63" s="29"/>
-      <c r="C63" s="29"/>
-      <c r="D63" s="34"/>
+      <c r="A63" s="31"/>
+      <c r="B63" s="31"/>
+      <c r="C63" s="31"/>
+      <c r="D63" s="36"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="29"/>
-      <c r="B64" s="29"/>
-      <c r="C64" s="29"/>
-      <c r="D64" s="34"/>
+      <c r="A64" s="31"/>
+      <c r="B64" s="31"/>
+      <c r="C64" s="31"/>
+      <c r="D64" s="36"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="29"/>
-      <c r="B65" s="29"/>
-      <c r="C65" s="29"/>
-      <c r="D65" s="34"/>
+      <c r="A65" s="31"/>
+      <c r="B65" s="31"/>
+      <c r="C65" s="31"/>
+      <c r="D65" s="36"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="29"/>
-      <c r="B66" s="29"/>
-      <c r="C66" s="29"/>
-      <c r="D66" s="34"/>
+      <c r="A66" s="31"/>
+      <c r="B66" s="31"/>
+      <c r="C66" s="31"/>
+      <c r="D66" s="36"/>
     </row>
     <row r="67" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="13"/>
@@ -5770,7 +5820,7 @@
       <c r="B77" s="1"/>
     </row>
     <row r="78" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="35"/>
+      <c r="A78" s="37"/>
       <c r="B78" s="1"/>
     </row>
     <row r="79" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>